<commit_message>
Add 2025-2026 season data and handle unplayed matches
- Teams: add Paperilla Parempi (36), Hot Wings (37), Tabula Rasa (38)
- Competitions: add P-S Harraste A (28, sarja) and P-S Harraste A
  playoff (29) for season 2025-2026
- Matches: append 14 rows (match_id 157-170): 12 regular-season games,
  semifinal vs VesKi (24.3.2026, 4-3 VL) and final vs NahU (11.4.2026).
  Final stored with empty goals pending today's game result.
- model.enrich_matches: treat matches with NaN goals as unplayed so
  outcome/goals_for/goals_against/points_from_match all become None.
  Previously the final was miscounted as a draw worth 1 point.

Current 2025-2026 record (13 played): 7-2-4, 69-61, 16 pts.
</commit_message>
<xml_diff>
--- a/mailajoket_2014_2026_dataworkbook.xlsx
+++ b/mailajoket_2014_2026_dataworkbook.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seasons" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TeamAliases" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matches" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standings" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rosters" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerSeasonStats" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Seasons" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Teams" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TeamAliases" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Competitions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Matches" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Standings" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Players" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Rosters" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="PlayerSeasonStats" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Seasons'!$A$1:$E$1</definedName>
@@ -7238,7 +7238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7828,6 +7828,51 @@
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Paperilla Parempi</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>paperilla-parempi</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Hot Wings</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>hot-wings</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Tabula Rasa</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>tabula-rasa</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
@@ -7929,7 +7974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8691,6 +8736,56 @@
       <c r="F28" s="4" t="inlineStr">
         <is>
           <t>2024-2025:p-s-harraste-a-sijoitusottelut:sijoitusottelut:</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>P-S Harraste A</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>sarja</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2025-2026:p-s-harraste-a:sarja:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>P-S Harraste A playoff</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>playoff</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2025-2026:p-s-harraste-a-playoff:playoff:</t>
         </is>
       </c>
     </row>
@@ -8709,7 +8804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J157"/>
+  <dimension ref="A1:J171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13463,6 +13558,495 @@
         </is>
       </c>
       <c r="J157" s="4" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>28</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>2025-10-19</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>30</v>
+      </c>
+      <c r="F158" t="n">
+        <v>20</v>
+      </c>
+      <c r="G158" t="n">
+        <v>2</v>
+      </c>
+      <c r="H158" t="n">
+        <v>2</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>otteluid:37850</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>28</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>2025-10-26</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>20</v>
+      </c>
+      <c r="F159" t="n">
+        <v>36</v>
+      </c>
+      <c r="G159" t="n">
+        <v>5</v>
+      </c>
+      <c r="H159" t="n">
+        <v>4</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>otteluid:37854</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>28</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>2025-11-09</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>37</v>
+      </c>
+      <c r="F160" t="n">
+        <v>20</v>
+      </c>
+      <c r="G160" t="n">
+        <v>6</v>
+      </c>
+      <c r="H160" t="n">
+        <v>3</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>otteluid:37855</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>28</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>18</v>
+      </c>
+      <c r="F161" t="n">
+        <v>20</v>
+      </c>
+      <c r="G161" t="n">
+        <v>2</v>
+      </c>
+      <c r="H161" t="n">
+        <v>12</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>otteluid:37863</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>28</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>20</v>
+      </c>
+      <c r="F162" t="n">
+        <v>13</v>
+      </c>
+      <c r="G162" t="n">
+        <v>5</v>
+      </c>
+      <c r="H162" t="n">
+        <v>5</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>otteluid:37859</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>28</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>20</v>
+      </c>
+      <c r="F163" t="n">
+        <v>38</v>
+      </c>
+      <c r="G163" t="n">
+        <v>3</v>
+      </c>
+      <c r="H163" t="n">
+        <v>7</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>otteluid:38711</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>28</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>33</v>
+      </c>
+      <c r="F164" t="n">
+        <v>20</v>
+      </c>
+      <c r="G164" t="n">
+        <v>4</v>
+      </c>
+      <c r="H164" t="n">
+        <v>5</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>otteluid:53873</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>28</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>20</v>
+      </c>
+      <c r="F165" t="n">
+        <v>16</v>
+      </c>
+      <c r="G165" t="n">
+        <v>9</v>
+      </c>
+      <c r="H165" t="n">
+        <v>4</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>otteluid:53872</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>28</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>20</v>
+      </c>
+      <c r="F166" t="n">
+        <v>37</v>
+      </c>
+      <c r="G166" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" t="n">
+        <v>8</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>otteluid:53875</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>28</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>20</v>
+      </c>
+      <c r="F167" t="n">
+        <v>38</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="n">
+        <v>6</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>otteluid:53891</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>28</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>20</v>
+      </c>
+      <c r="F168" t="n">
+        <v>21</v>
+      </c>
+      <c r="G168" t="n">
+        <v>10</v>
+      </c>
+      <c r="H168" t="n">
+        <v>5</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>otteluid:53886</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>28</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>36</v>
+      </c>
+      <c r="F169" t="n">
+        <v>20</v>
+      </c>
+      <c r="G169" t="n">
+        <v>5</v>
+      </c>
+      <c r="H169" t="n">
+        <v>11</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>otteluid:53889</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>29</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>20</v>
+      </c>
+      <c r="F170" t="n">
+        <v>33</v>
+      </c>
+      <c r="G170" t="n">
+        <v>4</v>
+      </c>
+      <c r="H170" t="n">
+        <v>3</v>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>VL</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>otteluid:55818;välierä</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>29</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>20</v>
+      </c>
+      <c r="F171" t="n">
+        <v>21</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>otteluid:56162;finaali - täydennetään</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>

</xml_diff>